<commit_message>
Ultima update del dia - Archivos retocados
</commit_message>
<xml_diff>
--- a/paginas.xlsx
+++ b/paginas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\ChambaGPT-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2389C4F-2B4F-4628-986D-FDB935E12A48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4937E74-08DB-4379-84C5-4DAF7CDD2A3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14595" tabRatio="704" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14595" tabRatio="704" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Learning" sheetId="8" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="235">
   <si>
     <t>ID</t>
   </si>
@@ -623,9 +623,6 @@
     <t>https://www.talent.com</t>
   </si>
   <si>
-    <t>https://hired.com</t>
-  </si>
-  <si>
     <t>https://www.toptal.com</t>
   </si>
   <si>
@@ -714,6 +711,30 @@
   </si>
   <si>
     <t>https://www.themuse.com/advice</t>
+  </si>
+  <si>
+    <t>https://www.lhh.com/es-mx/candidatos</t>
+  </si>
+  <si>
+    <t>🥈 VIBE TECH (Prestigio y Remoto Real / Corporativo de Élite)</t>
+  </si>
+  <si>
+    <t>https://www.adecco.com/es-mx/aspirantes</t>
+  </si>
+  <si>
+    <t>SITUACIÓN: Entras buscando “oportunidades” y sales con tres entrevistas para puestos operativos que no recuerdas haber aplicado. Prometen eficiencia, procesos pulidos y “talento adecuado”, pero la experiencia suele sentirse como una línea de ensamblaje donde tú eres la pieza intercambiable. Ideal si quieres volumen, rapidez y cero sorpresas emocionales.</t>
+  </si>
+  <si>
+    <t>Reclutamiento Masivo, Tradicional, Agencia</t>
+  </si>
+  <si>
+    <t>💀 GHOSTING PRO (Agregadores de Volumen / Reclutamiento Masivo)</t>
+  </si>
+  <si>
+    <t>Adecco</t>
+  </si>
+  <si>
+    <t>LLH</t>
   </si>
 </sst>
 </file>
@@ -869,7 +890,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -923,27 +944,25 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="9">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -961,6 +980,21 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1101,8 +1135,8 @@
     <tableColumn id="6" xr3:uid="{0C5DCD66-F23F-485C-B1CF-762876EFA25A}" name="Descripción (Original)" dataDxfId="4"/>
     <tableColumn id="4" xr3:uid="{6CD74F86-E237-48C5-BF40-E73EE24DE8E9}" name="Categoría" dataDxfId="3"/>
     <tableColumn id="5" xr3:uid="{899BF151-5354-4A9F-8DBF-AD66322FA351}" name="Palabras Clave / Tags" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{89EFBE11-F6C2-446F-B934-DBC3B5DA7D43}" name="URL" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{3F4B7804-E2E3-4932-973F-ADD50CC766D3}" name="Imagen" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{89EFBE11-F6C2-446F-B934-DBC3B5DA7D43}" name="URL" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{3F4B7804-E2E3-4932-973F-ADD50CC766D3}" name="Imagen" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1261,7 +1295,7 @@
         <v>40</v>
       </c>
       <c r="F2" s="27" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G2" s="18"/>
     </row>
@@ -1282,11 +1316,11 @@
         <v>61</v>
       </c>
       <c r="F3" s="27" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G3" s="13"/>
     </row>
-    <row r="4" spans="1:7" ht="25.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="63.75" x14ac:dyDescent="0.35">
       <c r="A4" s="14">
         <v>18</v>
       </c>
@@ -1303,7 +1337,7 @@
         <v>75</v>
       </c>
       <c r="F4" s="27" t="s">
-        <v>197</v>
+        <v>227</v>
       </c>
       <c r="G4" s="18"/>
     </row>
@@ -1370,7 +1404,7 @@
         <v>87</v>
       </c>
       <c r="F7" s="28" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="G7" s="13"/>
     </row>
@@ -1430,7 +1464,7 @@
         <v>103</v>
       </c>
       <c r="F2" s="27" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G2" s="3"/>
     </row>
@@ -1451,7 +1485,7 @@
         <v>105</v>
       </c>
       <c r="F3" s="27" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>5</v>
@@ -1474,7 +1508,7 @@
         <v>53</v>
       </c>
       <c r="F4" s="27" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G4" s="3"/>
     </row>
@@ -1495,7 +1529,7 @@
         <v>55</v>
       </c>
       <c r="F5" s="27" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>5</v>
@@ -1518,7 +1552,7 @@
         <v>57</v>
       </c>
       <c r="F6" s="27" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>5</v>
@@ -1541,7 +1575,7 @@
         <v>59</v>
       </c>
       <c r="F7" s="27" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G7" s="3"/>
     </row>
@@ -1562,7 +1596,7 @@
         <v>77</v>
       </c>
       <c r="F8" s="27" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>5</v>
@@ -1585,7 +1619,7 @@
         <v>97</v>
       </c>
       <c r="F9" s="27" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G9" s="3"/>
     </row>
@@ -1606,7 +1640,7 @@
         <v>99</v>
       </c>
       <c r="F10" s="27" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G10" s="3"/>
     </row>
@@ -1669,7 +1703,7 @@
         <v>45</v>
       </c>
       <c r="F2" s="27" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G2" s="18" t="s">
         <v>5</v>
@@ -1692,7 +1726,7 @@
         <v>69</v>
       </c>
       <c r="F3" s="27" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G3" s="18"/>
     </row>
@@ -1713,7 +1747,7 @@
         <v>95</v>
       </c>
       <c r="F4" s="27" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G4" s="13"/>
     </row>
@@ -1734,7 +1768,7 @@
         <v>140</v>
       </c>
       <c r="F5" s="27" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G5" s="18"/>
     </row>
@@ -1872,7 +1906,7 @@
         <v>145</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G6" s="13"/>
     </row>
@@ -1893,7 +1927,7 @@
         <v>147</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G7" s="18"/>
     </row>
@@ -1914,7 +1948,7 @@
         <v>148</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G8" s="13"/>
     </row>
@@ -1935,7 +1969,7 @@
         <v>149</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G9" s="18"/>
     </row>
@@ -1956,7 +1990,7 @@
         <v>143</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G10" s="18"/>
     </row>
@@ -1988,14 +2022,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6615E48-7057-414B-8352-E4310E9023F0}">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="5" max="5" width="34.1328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="32" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="25.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
@@ -2018,7 +2052,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="25.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A2" s="9">
         <v>14</v>
       </c>
@@ -2041,7 +2075,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" s="14">
         <v>2</v>
       </c>
@@ -2062,196 +2096,245 @@
       </c>
       <c r="G3" s="18"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="9">
+        <v>4</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>188</v>
+      </c>
+      <c r="G4" s="13"/>
+    </row>
+    <row r="5" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="14">
+        <v>13</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>189</v>
+      </c>
+      <c r="G5" s="18"/>
+    </row>
+    <row r="6" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="14">
+        <v>17</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="G6" s="18" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A7" s="14">
+        <v>18</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>234</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7" s="32" t="s">
+        <v>228</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="F7" s="35" t="s">
+        <v>227</v>
+      </c>
+      <c r="G7" s="37"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A8" s="9">
         <v>22</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B8" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C8" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D8" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E8" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F8" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="G4" s="13"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="9">
+      <c r="G8" s="13"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A9" s="9">
         <v>36</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B9" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C9" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D9" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E9" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="F9" s="12" t="s">
         <v>194</v>
       </c>
-      <c r="G5" s="13"/>
-    </row>
-    <row r="6" spans="1:7" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="9">
+      <c r="G9" s="13"/>
+    </row>
+    <row r="10" spans="1:16" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="9">
         <v>37</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B10" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C10" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D10" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E10" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="F10" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="G6" s="13"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="9">
-        <v>4</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="11" t="s">
+      <c r="G10" s="13"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A11" s="31">
         <v>48</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>188</v>
-      </c>
-      <c r="G7" s="13"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="9">
-        <v>48</v>
-      </c>
-      <c r="B8" s="10" t="s">
+      <c r="B11" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C11" s="33" t="s">
         <v>125</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D11" s="34" t="s">
         <v>177</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E11" s="34" t="s">
         <v>153</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F11" s="36" t="s">
         <v>139</v>
       </c>
-      <c r="G8" s="13"/>
-    </row>
-    <row r="9" spans="1:7" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="14">
-        <v>13</v>
-      </c>
-      <c r="B9" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>167</v>
-      </c>
-      <c r="E9" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="F9" s="17" t="s">
-        <v>189</v>
-      </c>
-      <c r="G9" s="18"/>
-    </row>
-    <row r="10" spans="1:7" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="14">
-        <v>17</v>
-      </c>
-      <c r="B10" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="E10" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="F10" s="17" t="s">
-        <v>190</v>
-      </c>
-      <c r="G10" s="18" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11">
+      <c r="G11" s="36"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A12">
         <v>50</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>179</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C12" t="s">
         <v>180</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D12" t="s">
         <v>176</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E12" t="s">
         <v>181</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F12" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A13" s="30">
         <v>51</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" s="32" t="s">
         <v>182</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C13" s="32" t="s">
         <v>183</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D13" t="s">
         <v>177</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E13" s="32" t="s">
         <v>184</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F13" t="s">
         <v>192</v>
       </c>
+      <c r="M13" s="17"/>
+      <c r="P13" s="18"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A14" s="31">
+        <v>52</v>
+      </c>
+      <c r="B14" t="s">
+        <v>233</v>
+      </c>
+      <c r="C14" t="s">
+        <v>230</v>
+      </c>
+      <c r="D14" t="s">
+        <v>232</v>
+      </c>
+      <c r="E14" t="s">
+        <v>231</v>
+      </c>
+      <c r="F14" s="29" t="s">
+        <v>229</v>
+      </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:G14">
+    <sortCondition ref="A2:A14"/>
+  </sortState>
+  <hyperlinks>
+    <hyperlink ref="F14" r:id="rId1" xr:uid="{350D35D9-6428-47C2-ACC9-7D94D729949F}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2301,7 +2384,7 @@
         <v>51</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G2" s="18"/>
     </row>
@@ -2322,7 +2405,7 @@
         <v>49</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G3" s="13"/>
     </row>
@@ -2343,7 +2426,7 @@
         <v>81</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G4" s="18"/>
     </row>
@@ -2364,7 +2447,7 @@
         <v>71</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G5" s="18"/>
     </row>
@@ -2385,7 +2468,7 @@
         <v>89</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G6" s="18"/>
     </row>
@@ -2406,7 +2489,7 @@
         <v>93</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G7" s="13"/>
     </row>
@@ -2427,7 +2510,7 @@
         <v>63</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="G8" s="13"/>
     </row>
@@ -2448,7 +2531,7 @@
         <v>101</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G9" s="3"/>
     </row>
@@ -2469,7 +2552,7 @@
         <v>91</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G10" s="3"/>
     </row>

</xml_diff>